<commit_message>
ajout collection projet et finalisation
</commit_message>
<xml_diff>
--- a/public/documents/tableau.xlsx
+++ b/public/documents/tableau.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thedr\Documents\Sio_1ere_annee\Tableau pour portfolio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dev\portfolio\public\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDC6B8C-AEE7-4FCC-93FF-3F17ABCA0896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9985A8-9E47-4C90-A78B-DBC44080A67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$34</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -127,9 +127,6 @@
     <t>X</t>
   </si>
   <si>
-    <t>15/09/25 au 31/10/25</t>
-  </si>
-  <si>
     <t>03/11/25 au 12/12/25</t>
   </si>
   <si>
@@ -155,24 +152,6 @@
   </si>
   <si>
     <t xml:space="preserve">Centre de formation : Ifide SUP- Formation Eckbolsheim </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Application Web de gestion de tâches — PHP / MySQL (MAMP)
-• MCD / MLD et script SQL de création de la BDD
-• Connexion PDO et requêtes préparées (anti-injection SQL)
-• CRUD complet : création, lecture, modification, suppression
-• Validation JavaScript des saisies côté client
-• Échappement htmlspecialchars contre les XSS
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TP Gestion d'une collection — PHP / MySQL multi-tables
-• MCD à 4 tables liées et schéma relationnel
-• Requêtes JOIN et LEFT JOIN (extraits commentés)
-• CRUD multi-entités sur plusieurs types d'objets
-• Architecture modulaire (header / footer / navigation via require)
-• Jeu d'essai et résultats de tests
-</t>
   </si>
   <si>
     <t xml:space="preserve">Projet AP2 « Parcus » — Infrastructure réseau d'un par informatique sur VM
@@ -229,6 +208,15 @@
 • Tests
 • Mise a jour et optimisation UI/UX
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TP Gestion d'une collection — PHP / MySQL multi-tables
+• MCD à 4 tables liées et schéma relationnel
+• Requêtes JOIN et LEFT JOIN (extraits commentés)
+• CRUD complet : création, lecture, modification, suppression
+• Architecture modulaire (header / footer / navigation via require)
+• Jeu d'essai et résultats de tests
+• Échappement htmlspecialchars contre les XSS, hashage MDP </t>
   </si>
 </sst>
 </file>
@@ -635,6 +623,15 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -652,15 +649,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -930,67 +918,67 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.81640625" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AQ34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="77.1796875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="29.08984375" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7265625" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.453125" customWidth="1"/>
-    <col min="44" max="16384" width="10.81640625" style="1"/>
+    <col min="1" max="1" width="77.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.42578125" customWidth="1"/>
+    <col min="44" max="16384" width="10.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="28"/>
-    </row>
-    <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="H1" s="22"/>
+    </row>
+    <row r="2" spans="1:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-    </row>
-    <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+    </row>
+    <row r="3" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="30" t="s">
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
+    <row r="4" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
       <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
@@ -1001,23 +989,23 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+    <row r="5" spans="1:13" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-    </row>
-    <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25" t="s">
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+    </row>
+    <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="29" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -1039,9 +1027,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="9" customFormat="1" ht="324.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="25"/>
-      <c r="B7" s="26"/>
+    <row r="7" spans="1:13" s="9" customFormat="1" ht="324.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="28"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="7" t="s">
         <v>17</v>
       </c>
@@ -1061,21 +1049,21 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="27" t="s">
+    <row r="8" spans="1:13" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-    </row>
-    <row r="9" spans="1:13" s="9" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+    </row>
+    <row r="9" spans="1:13" s="9" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B9" s="11" t="s">
         <v>24</v>
@@ -1091,9 +1079,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="9" customFormat="1" ht="140" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" s="9" customFormat="1" ht="126.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>26</v>
@@ -1106,14 +1094,12 @@
       <c r="F10" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="G10" s="13" t="s">
-        <v>25</v>
-      </c>
+      <c r="G10" s="13"/>
       <c r="H10" s="14"/>
     </row>
-    <row r="11" spans="1:13" s="9" customFormat="1" ht="127" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" s="9" customFormat="1" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>27</v>
@@ -1121,17 +1107,21 @@
       <c r="C11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="13"/>
+      <c r="D11" s="13" t="s">
+        <v>25</v>
+      </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="13"/>
+      <c r="G11" s="13" t="s">
+        <v>25</v>
+      </c>
       <c r="H11" s="14"/>
     </row>
-    <row r="12" spans="1:13" s="9" customFormat="1" ht="136.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" s="9" customFormat="1" ht="101.45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>28</v>
@@ -1139,53 +1129,41 @@
       <c r="C12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="13" t="s">
-        <v>25</v>
-      </c>
+      <c r="D12" s="13"/>
       <c r="E12" s="13"/>
       <c r="F12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="13" t="s">
-        <v>25</v>
-      </c>
+      <c r="G12" s="13"/>
       <c r="H12" s="14"/>
     </row>
-    <row r="13" spans="1:13" s="9" customFormat="1" ht="101.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" s="9" customFormat="1" ht="135" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="13" t="s">
-        <v>25</v>
-      </c>
+      <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
-      <c r="F13" s="13" t="s">
-        <v>25</v>
-      </c>
+      <c r="F13" s="13"/>
       <c r="G13" s="13"/>
-      <c r="H13" s="14"/>
-    </row>
-    <row r="14" spans="1:13" s="9" customFormat="1" ht="135" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>30</v>
-      </c>
+      <c r="H13" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="10"/>
+      <c r="B14" s="11"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
-      <c r="H14" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H14" s="14"/>
+    </row>
+    <row r="15" spans="1:13" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10"/>
       <c r="B15" s="11"/>
       <c r="C15" s="13"/>
@@ -1195,7 +1173,7 @@
       <c r="G15" s="13"/>
       <c r="H15" s="14"/>
     </row>
-    <row r="16" spans="1:13" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10"/>
       <c r="B16" s="11"/>
       <c r="C16" s="13"/>
@@ -1205,7 +1183,7 @@
       <c r="G16" s="13"/>
       <c r="H16" s="14"/>
     </row>
-    <row r="17" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="10"/>
       <c r="B17" s="11"/>
       <c r="C17" s="13"/>
@@ -1215,73 +1193,73 @@
       <c r="G17" s="13"/>
       <c r="H17" s="14"/>
     </row>
-    <row r="18" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="14"/>
-    </row>
-    <row r="19" spans="1:8" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+    <row r="18" spans="1:8" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="25"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
+    </row>
+    <row r="19" spans="1:8" s="9" customFormat="1" ht="160.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-    </row>
-    <row r="20" spans="1:8" s="9" customFormat="1" ht="160.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="H19" s="14"/>
+    </row>
+    <row r="20" spans="1:8" s="9" customFormat="1" ht="181.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B20" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13" t="s">
+        <v>25</v>
+      </c>
       <c r="F20" s="13" t="s">
         <v>25</v>
       </c>
       <c r="G20" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="H20" s="14"/>
-    </row>
-    <row r="21" spans="1:8" s="9" customFormat="1" ht="181.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>33</v>
-      </c>
+      <c r="H20" s="14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="10"/>
+      <c r="B21" s="11"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="14"/>
+    </row>
+    <row r="22" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="10"/>
       <c r="B22" s="11"/>
       <c r="C22" s="13"/>
@@ -1291,7 +1269,7 @@
       <c r="G22" s="13"/>
       <c r="H22" s="14"/>
     </row>
-    <row r="23" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="10"/>
       <c r="B23" s="11"/>
       <c r="C23" s="13"/>
@@ -1301,7 +1279,7 @@
       <c r="G23" s="13"/>
       <c r="H23" s="14"/>
     </row>
-    <row r="24" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="10"/>
       <c r="B24" s="11"/>
       <c r="C24" s="13"/>
@@ -1311,7 +1289,7 @@
       <c r="G24" s="13"/>
       <c r="H24" s="14"/>
     </row>
-    <row r="25" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="10"/>
       <c r="B25" s="11"/>
       <c r="C25" s="13"/>
@@ -1321,29 +1299,29 @@
       <c r="G25" s="13"/>
       <c r="H25" s="14"/>
     </row>
-    <row r="26" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
-      <c r="H26" s="14"/>
-    </row>
-    <row r="27" spans="1:8" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-    </row>
-    <row r="28" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" s="9" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+    </row>
+    <row r="27" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="10"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="14"/>
+    </row>
+    <row r="28" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10"/>
       <c r="B28" s="11"/>
       <c r="C28" s="13"/>
@@ -1353,7 +1331,7 @@
       <c r="G28" s="13"/>
       <c r="H28" s="14"/>
     </row>
-    <row r="29" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10"/>
       <c r="B29" s="11"/>
       <c r="C29" s="13"/>
@@ -1363,7 +1341,7 @@
       <c r="G29" s="13"/>
       <c r="H29" s="14"/>
     </row>
-    <row r="30" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10"/>
       <c r="B30" s="11"/>
       <c r="C30" s="13"/>
@@ -1373,7 +1351,7 @@
       <c r="G30" s="13"/>
       <c r="H30" s="14"/>
     </row>
-    <row r="31" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="10"/>
       <c r="B31" s="11"/>
       <c r="C31" s="13"/>
@@ -1383,7 +1361,7 @@
       <c r="G31" s="13"/>
       <c r="H31" s="14"/>
     </row>
-    <row r="32" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="10"/>
       <c r="B32" s="11"/>
       <c r="C32" s="13"/>
@@ -1393,50 +1371,40 @@
       <c r="G32" s="13"/>
       <c r="H32" s="14"/>
     </row>
-    <row r="33" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="13"/>
-      <c r="H33" s="14"/>
-    </row>
-    <row r="34" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="15"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="18"/>
-    </row>
-    <row r="35" spans="1:8" s="9" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="19"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
-      <c r="G35" s="21"/>
-      <c r="H35" s="21"/>
+    <row r="33" spans="1:8" s="9" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="15"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="18"/>
+    </row>
+    <row r="34" spans="1:8" s="9" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="19"/>
+      <c r="B34" s="20"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A8:H8"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="F3:H3"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A8:H8"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>